<commit_message>
Add ability to specify total number of circuits for panel schedules
Update OCR parsing logic to accept an optional `number_of_ckts` parameter, defaulting to 18-80 even numbers. The Excel template is also updated to handle odd/even circuit layouts and extract more circuit parameters.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: db39287f-61a8-4c70-91e9-735e92f424ca
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/0e87c197-6493-4ee7-94fe-fe960b787501/db39287f-61a8-4c70-91e9-735e92f424ca/ANDp6DG
</commit_message>
<xml_diff>
--- a/templates/default_panelboard_template.xlsx
+++ b/templates/default_panelboard_template.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PP-1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:R50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>PP-1</t>
+          <t>PANEL NAME</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -436,6 +436,9 @@
       <c r="M1" t="inlineStr"/>
       <c r="N1" t="inlineStr"/>
       <c r="O1" t="inlineStr"/>
+      <c r="P1" t="inlineStr"/>
+      <c r="Q1" t="inlineStr"/>
+      <c r="R1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -454,21 +457,24 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOCATION:  </t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LOCATION:  </t>
-        </is>
-      </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
           <t>ELEC. EQUIP. PAD</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -489,21 +495,24 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FED FROM:  </t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FED FROM:  </t>
-        </is>
-      </c>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
           <t>MDP AND ATS #1</t>
         </is>
       </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -520,21 +529,24 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UL LISTED EQUIPMENT SHORT CIRCUIT RATING:  </t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UL LISTED EQUIPMENT SHORT CIRCUIT RATING:  </t>
-        </is>
-      </c>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
           <t>65K</t>
         </is>
       </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -553,21 +565,24 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MAXIMUM AVAILABLE SHORT CIRCUIT CURRENT:  </t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MAXIMUM AVAILABLE SHORT CIRCUIT CURRENT:  </t>
-        </is>
-      </c>
+      <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -586,21 +601,24 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PHASE CONDUCTOR:  </t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PHASE CONDUCTOR:  </t>
-        </is>
-      </c>
+      <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr">
         <is>
           <t>#4/0</t>
         </is>
       </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -619,21 +637,24 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NEUTRAL CONDUCTOR:  </t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NEUTRAL CONDUCTOR:  </t>
-        </is>
-      </c>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
           <t>#4/0</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -652,21 +673,24 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELECTRICAL GROUND CONDUCTOR:  </t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ELECTRICAL GROUND CONDUCTOR:  </t>
-        </is>
-      </c>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>#4</t>
         </is>
       </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -700,6 +724,9 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -737,6 +764,9 @@
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -814,6 +844,9 @@
           <t>LOAD DESCRIPTION &amp; LOCATION</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -859,6 +892,9 @@
           <t>GATE HOIST #13 MOTOR</t>
         </is>
       </c>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -881,13 +917,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>3</v>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>4</v>
+      </c>
       <c r="J13" t="n">
         <v>20</v>
       </c>
@@ -906,6 +946,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -928,13 +971,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>5</v>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>6</v>
+      </c>
       <c r="J14" t="n">
         <v>20</v>
       </c>
@@ -953,6 +1000,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -972,7 +1022,7 @@
         <v>20</v>
       </c>
       <c r="G15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -980,7 +1030,7 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J15" t="n">
         <v>20</v>
@@ -998,6 +1048,9 @@
           <t>SPARE</t>
         </is>
       </c>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1020,13 +1073,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>9</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>10</v>
+      </c>
       <c r="J16" t="n">
         <v>20</v>
       </c>
@@ -1043,6 +1100,9 @@
           <t>SPARE</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1065,13 +1125,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="n">
+        <v>11</v>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>12</v>
+      </c>
       <c r="J17" t="n">
         <v>20</v>
       </c>
@@ -1088,6 +1152,9 @@
           <t>CONTACTOR CONTROL CIRCUIT</t>
         </is>
       </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1107,7 +1174,7 @@
         <v>20</v>
       </c>
       <c r="G18" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1115,7 +1182,7 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="J18" t="n">
         <v>20</v>
@@ -1133,6 +1200,9 @@
           <t>GATE #9 HOIST MOTOR</t>
         </is>
       </c>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1155,13 +1225,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="n">
+        <v>15</v>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>16</v>
+      </c>
       <c r="J19" t="inlineStr">
         <is>
           <t>-</t>
@@ -1182,6 +1256,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1204,13 +1281,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>17</v>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>18</v>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
           <t>-</t>
@@ -1231,6 +1312,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1250,7 +1334,7 @@
         <v>20</v>
       </c>
       <c r="G21" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1258,7 +1342,7 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="J21" t="n">
         <v>20</v>
@@ -1276,6 +1360,9 @@
           <t>GATE #10 HOIST MOTOR</t>
         </is>
       </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1298,13 +1385,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>21</v>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>22</v>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
           <t>-</t>
@@ -1325,6 +1416,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1347,13 +1441,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>23</v>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>24</v>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
           <t>-</t>
@@ -1374,6 +1472,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1393,7 +1494,7 @@
         <v>20</v>
       </c>
       <c r="G24" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1401,7 +1502,7 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="J24" t="n">
         <v>20</v>
@@ -1419,6 +1520,9 @@
           <t>GATE #11 HOIST MOTOR</t>
         </is>
       </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1441,13 +1545,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>27</v>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="n">
+        <v>28</v>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
           <t>-</t>
@@ -1468,6 +1576,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1490,13 +1601,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>29</v>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
+      <c r="I26" t="n">
+        <v>30</v>
+      </c>
       <c r="J26" t="inlineStr">
         <is>
           <t>-</t>
@@ -1517,6 +1632,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1536,7 +1654,7 @@
         <v>20</v>
       </c>
       <c r="G27" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1544,7 +1662,7 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="J27" t="n">
         <v>20</v>
@@ -1562,6 +1680,9 @@
           <t>GATE #12 HOIST MOTOR</t>
         </is>
       </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1584,13 +1705,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" t="n">
+        <v>33</v>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
+      <c r="I28" t="n">
+        <v>34</v>
+      </c>
       <c r="J28" t="inlineStr">
         <is>
           <t>-</t>
@@ -1611,6 +1736,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1633,13 +1761,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="n">
+        <v>35</v>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
+      <c r="I29" t="n">
+        <v>36</v>
+      </c>
       <c r="J29" t="inlineStr">
         <is>
           <t>-</t>
@@ -1660,6 +1792,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1679,7 +1814,7 @@
         <v>20</v>
       </c>
       <c r="G30" t="n">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1687,7 +1822,7 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="J30" t="n">
         <v>20</v>
@@ -1705,6 +1840,9 @@
           <t>LIGHTING HOIST 1, 3, 5, 7, 9, 11, 13</t>
         </is>
       </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1727,13 +1865,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="n">
+        <v>39</v>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="n">
+        <v>40</v>
+      </c>
       <c r="J31" t="n">
         <v>20</v>
       </c>
@@ -1750,6 +1892,9 @@
           <t>LIGHTING HOIST 2, 4, 6, 8, 12, 12, 14</t>
         </is>
       </c>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1772,13 +1917,17 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="n">
+        <v>41</v>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" t="n">
+        <v>42</v>
+      </c>
       <c r="J32" t="n">
         <v>20</v>
       </c>
@@ -1795,431 +1944,257 @@
           <t>SPARE</t>
         </is>
       </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GATE #8 HOIST MOTOR</t>
+          <t>TOTAL AMPS</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>11</v>
-      </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="n">
-        <v>3</v>
-      </c>
-      <c r="F33" t="n">
-        <v>20</v>
-      </c>
-      <c r="G33" t="n">
-        <v>15</v>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>16</v>
-      </c>
-      <c r="J33" t="n">
-        <v>20</v>
-      </c>
-      <c r="K33" t="n">
-        <v>1</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="C33" t="n">
+        <v>77</v>
+      </c>
+      <c r="D33" t="n">
+        <v>77</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
+        <v>58</v>
+      </c>
+      <c r="M33" t="n">
+        <v>58</v>
+      </c>
+      <c r="N33" t="n">
+        <v>57</v>
+      </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>SPARE</t>
-        </is>
-      </c>
+          <t>TOTAL AMPS</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
-      <c r="C34" t="n">
-        <v>11</v>
-      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>PH. A</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="n">
-        <v>20</v>
-      </c>
-      <c r="K34" t="n">
-        <v>1</v>
-      </c>
+          <t>PH. B</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>PH. C</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>NOTES:</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
-      <c r="M34" t="n">
-        <v>0</v>
-      </c>
+      <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>SPARE</t>
-        </is>
-      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" t="n">
-        <v>11</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="n">
-        <v>20</v>
-      </c>
-      <c r="K35" t="n">
-        <v>1</v>
-      </c>
+          <t>TOTAL PHASE AMPS</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>135</v>
+      </c>
+      <c r="H35" t="n">
+        <v>135</v>
+      </c>
+      <c r="I35" t="n">
+        <v>134</v>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>SPARE</t>
-        </is>
-      </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>SPACE</t>
-        </is>
-      </c>
+      <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="n">
-        <v>3</v>
-      </c>
+      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TOTAL PHASE KVA</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>17</v>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+        <v>37.395</v>
+      </c>
+      <c r="H36" t="n">
+        <v>37.395</v>
       </c>
       <c r="I36" t="n">
-        <v>18</v>
-      </c>
-      <c r="J36" t="n">
-        <v>30</v>
-      </c>
-      <c r="K36" t="n">
-        <v>3</v>
-      </c>
-      <c r="L36" t="n">
-        <v>2</v>
-      </c>
+        <v>37.118</v>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>SPD</t>
-        </is>
-      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TOTAL 3-PHASE KVA</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="H37" t="n">
+        <v>111.908</v>
       </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
-      <c r="M37" t="n">
-        <v>2</v>
-      </c>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="n">
-        <v>2</v>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>SPACE</t>
-        </is>
-      </c>
+      <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="n">
-        <v>3</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>19</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I39" t="n">
-        <v>20</v>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K39" t="n">
-        <v>3</v>
-      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>SPACE</t>
-        </is>
-      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>TOTAL AMPS</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>88</v>
-      </c>
-      <c r="C42" t="n">
-        <v>88</v>
-      </c>
-      <c r="D42" t="n">
-        <v>88</v>
-      </c>
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
@@ -2227,20 +2202,13 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="n">
-        <v>60</v>
-      </c>
-      <c r="M42" t="n">
-        <v>60</v>
-      </c>
-      <c r="N42" t="n">
-        <v>59</v>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>TOTAL AMPS</t>
-        </is>
-      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
@@ -2249,31 +2217,18 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>PH. A</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>PH. B</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>PH. C</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>NOTES:</t>
-        </is>
-      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
@@ -2281,26 +2236,19 @@
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>TOTAL PHASE AMPS</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>148</v>
-      </c>
-      <c r="H44" t="n">
-        <v>148</v>
-      </c>
-      <c r="I44" t="n">
-        <v>147</v>
-      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
@@ -2308,26 +2256,19 @@
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>TOTAL PHASE KVA</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>40.996</v>
-      </c>
-      <c r="H45" t="n">
-        <v>40.996</v>
-      </c>
-      <c r="I45" t="n">
-        <v>40.719</v>
-      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
@@ -2335,15 +2276,9 @@
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>TOTAL 3-PHASE KVA</t>
-        </is>
-      </c>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" t="n">
-        <v>122.711</v>
-      </c>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
@@ -2351,6 +2286,89 @@
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>